<commit_message>
更新看板 10月16日 — KPI465.8万(27.1%) 净流水369.7万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,11 +488,11 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>5330</v>
+        <v>412222.01</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.4%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -500,20 +500,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1449.8%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-71945.45</v>
+        <v>334946.56</v>
       </c>
       <c r="I2" t="n">
-        <v>-67945</v>
+        <v>309763</v>
       </c>
       <c r="J2" t="n">
-        <v>-4000</v>
+        <v>25182</v>
       </c>
       <c r="K2" t="n">
-        <v>-60137</v>
+        <v>288372</v>
       </c>
     </row>
     <row r="3">
@@ -531,11 +531,11 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>1915</v>
+        <v>151062.99</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -543,20 +543,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9275.5%</t>
+          <t>117.6%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-175710.37</v>
+        <v>-26562.38</v>
       </c>
       <c r="I3" t="n">
-        <v>-170730</v>
+        <v>-22200</v>
       </c>
       <c r="J3" t="n">
-        <v>-4980</v>
+        <v>-4362</v>
       </c>
       <c r="K3" t="n">
-        <v>-157210</v>
+        <v>-9456</v>
       </c>
     </row>
     <row r="4">
@@ -574,11 +574,11 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>4837</v>
+        <v>447587.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -586,20 +586,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1962.1%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-90067.97</v>
+        <v>352682.91</v>
       </c>
       <c r="I4" t="n">
-        <v>-90067</v>
+        <v>352644</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="K4" t="n">
-        <v>-68067</v>
+        <v>264072</v>
       </c>
     </row>
     <row r="5">
@@ -617,11 +617,11 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>732</v>
+        <v>623184.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>38.9%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -629,20 +629,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>32239.9%</t>
+          <t>37.9%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>-235263.88</v>
+        <v>387188.48</v>
       </c>
       <c r="I5" t="n">
-        <v>-233283</v>
+        <v>294568</v>
       </c>
       <c r="J5" t="n">
-        <v>-1980</v>
+        <v>92620</v>
       </c>
       <c r="K5" t="n">
-        <v>-165223</v>
+        <v>181958</v>
       </c>
     </row>
     <row r="6">
@@ -660,11 +660,11 @@
         <v>2500000</v>
       </c>
       <c r="D6" t="n">
-        <v>752468.0199999999</v>
+        <v>799979.9199999999</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -672,20 +672,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>704668.0199999999</v>
+        <v>752179.9199999999</v>
       </c>
       <c r="I6" t="n">
-        <v>287059</v>
+        <v>317573</v>
       </c>
       <c r="J6" t="n">
-        <v>417608</v>
+        <v>434606</v>
       </c>
       <c r="K6" t="n">
-        <v>715668</v>
+        <v>722383</v>
       </c>
     </row>
     <row r="7">
@@ -703,11 +703,11 @@
         <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>38</v>
+        <v>79501.84</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -715,20 +715,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>14360.5%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>-5419</v>
+        <v>74044.84</v>
       </c>
       <c r="I7" t="n">
-        <v>-19</v>
+        <v>56843</v>
       </c>
       <c r="J7" t="n">
-        <v>-5400</v>
+        <v>17201</v>
       </c>
       <c r="K7" t="n">
-        <v>-19</v>
+        <v>18868</v>
       </c>
     </row>
     <row r="8">
@@ -746,11 +746,11 @@
         <v>600000</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>308810</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -758,20 +758,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.9%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>-2680</v>
+        <v>306130</v>
       </c>
       <c r="I8" t="n">
-        <v>-1680</v>
+        <v>28540</v>
       </c>
       <c r="J8" t="n">
-        <v>-1000</v>
+        <v>277590</v>
       </c>
       <c r="K8" t="n">
-        <v>-1680</v>
+        <v>51156</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>22337.55</v>
+        <v>253609.03</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>147.7%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>-10662.45</v>
+        <v>220609.03</v>
       </c>
       <c r="I9" t="n">
-        <v>-17000</v>
+        <v>54335</v>
       </c>
       <c r="J9" t="n">
-        <v>-16000</v>
+        <v>143936</v>
       </c>
       <c r="K9" t="n">
-        <v>22337</v>
+        <v>33633</v>
       </c>
     </row>
     <row r="10">
@@ -832,11 +832,11 @@
         <v>1100000</v>
       </c>
       <c r="D10" t="n">
-        <v>6383.9</v>
+        <v>69335.91</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.6%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -844,20 +844,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1751.1%</t>
+          <t>161.2%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>-105404.1</v>
+        <v>-42452.09</v>
       </c>
       <c r="I10" t="n">
-        <v>-58580</v>
+        <v>-51212</v>
       </c>
       <c r="J10" t="n">
-        <v>-53179</v>
+        <v>2405</v>
       </c>
       <c r="K10" t="n">
-        <v>-37204</v>
+        <v>-31634</v>
       </c>
     </row>
     <row r="11">
@@ -875,11 +875,11 @@
         <v>400000</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>45281</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -887,20 +887,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>37480.7%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>-7102.33</v>
+        <v>38159.67</v>
       </c>
       <c r="I11" t="n">
-        <v>-7102</v>
+        <v>-5794</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>43954</v>
       </c>
       <c r="K11" t="n">
-        <v>-19</v>
+        <v>3455</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>500000</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>241031</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>48.2%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-10419</v>
+        <v>230612</v>
       </c>
       <c r="I12" t="n">
-        <v>-19</v>
+        <v>53422</v>
       </c>
       <c r="J12" t="n">
-        <v>-10400</v>
+        <v>177190</v>
       </c>
       <c r="K12" t="n">
-        <v>-19</v>
+        <v>91438</v>
       </c>
     </row>
     <row r="13">
@@ -961,11 +961,11 @@
         <v>1900000</v>
       </c>
       <c r="D13" t="n">
-        <v>22918.8</v>
+        <v>131164.8</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -973,20 +973,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>11724.8</v>
+        <v>119970.8</v>
       </c>
       <c r="I13" t="n">
-        <v>-796</v>
+        <v>14424</v>
       </c>
       <c r="J13" t="n">
-        <v>-10398</v>
+        <v>82628</v>
       </c>
       <c r="K13" t="n">
-        <v>21724</v>
+        <v>39912</v>
       </c>
     </row>
     <row r="14">
@@ -1004,11 +1004,11 @@
         <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>22868.59</v>
+        <v>744132.1000000001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2.3%</t>
+          <t>74.4%</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1016,20 +1016,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>435.9%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>-76820</v>
+        <v>644443.5100000001</v>
       </c>
       <c r="I14" t="n">
-        <v>-67920</v>
+        <v>76426</v>
       </c>
       <c r="J14" t="n">
-        <v>-30100</v>
+        <v>546816</v>
       </c>
       <c r="K14" t="n">
-        <v>-46720</v>
+        <v>285975</v>
       </c>
     </row>
     <row r="15">
@@ -1047,11 +1047,11 @@
         <v>900000</v>
       </c>
       <c r="D15" t="n">
-        <v>39430.85</v>
+        <v>266321.85</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1059,20 +1059,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>85.2%</t>
+          <t>12.6%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5821.849999999999</v>
+        <v>232712.85</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>59105</v>
       </c>
       <c r="J15" t="n">
-        <v>-33600</v>
+        <v>134186</v>
       </c>
       <c r="K15" t="n">
-        <v>39421</v>
+        <v>41134</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>638</v>
+        <v>85190</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>989.7%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>-5676</v>
+        <v>78876</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>32053</v>
       </c>
       <c r="J16" t="n">
-        <v>-5676</v>
+        <v>46823</v>
       </c>
       <c r="K16" t="n">
-        <v>-1680</v>
+        <v>9202</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
更新看板 10月19日 — KPI350.2万(20.4%) 净流水211.1万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>518692.01</v>
+        <v>224627</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>35.8%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>77934.45</v>
+        <v>80794.45</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>440757.56</v>
+        <v>143832.55</v>
       </c>
       <c r="I2" t="n">
-        <v>415555</v>
+        <v>145975</v>
       </c>
       <c r="J2" t="n">
-        <v>25201</v>
+        <v>-2143</v>
       </c>
       <c r="K2" t="n">
-        <v>392989</v>
+        <v>154446</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>191734.13</v>
+        <v>102457.42</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>179454.37</v>
+        <v>182952.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>93.6%</t>
+          <t>178.6%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>12279.76000000001</v>
+        <v>-80494.65000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>-3369</v>
+        <v>-97792</v>
       </c>
       <c r="J3" t="n">
-        <v>15649</v>
+        <v>17297</v>
       </c>
       <c r="K3" t="n">
-        <v>28787</v>
+        <v>-62592</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>558937.88</v>
+        <v>272865</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>39.9%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>99419.97</v>
+        <v>110888.97</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>40.6%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>459517.91</v>
+        <v>161976.03</v>
       </c>
       <c r="I4" t="n">
-        <v>459460</v>
+        <v>161938</v>
       </c>
       <c r="J4" t="n">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="K4" t="n">
-        <v>306709</v>
+        <v>118982</v>
       </c>
     </row>
     <row r="5">
@@ -617,32 +617,32 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1075132.36</v>
+        <v>799874</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>67.2%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>235995.88</v>
+        <v>262558.54</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>32.8%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>839136.4799999999</v>
+        <v>537315.46</v>
       </c>
       <c r="I5" t="n">
-        <v>661205</v>
+        <v>393979</v>
       </c>
       <c r="J5" t="n">
-        <v>177931</v>
+        <v>143336</v>
       </c>
       <c r="K5" t="n">
-        <v>582106</v>
+        <v>503795</v>
       </c>
     </row>
     <row r="6">
@@ -660,32 +660,32 @@
         <v>2500000</v>
       </c>
       <c r="D6" t="n">
-        <v>976484.92</v>
+        <v>966033.92</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>38.6%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>47800</v>
+        <v>58819</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4.9%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>928684.92</v>
+        <v>907214.92</v>
       </c>
       <c r="I6" t="n">
-        <v>377437</v>
+        <v>337218</v>
       </c>
       <c r="J6" t="n">
-        <v>551247</v>
+        <v>569996</v>
       </c>
       <c r="K6" t="n">
-        <v>888490</v>
+        <v>908816</v>
       </c>
     </row>
     <row r="7">
@@ -703,11 +703,11 @@
         <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>81817.84</v>
+        <v>14276</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -715,20 +715,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>38.2%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>76360.84</v>
+        <v>8819</v>
       </c>
       <c r="I7" t="n">
-        <v>57279</v>
+        <v>11939</v>
       </c>
       <c r="J7" t="n">
-        <v>18881</v>
+        <v>-3320</v>
       </c>
       <c r="K7" t="n">
-        <v>20786</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="8">
@@ -746,11 +746,11 @@
         <v>600000</v>
       </c>
       <c r="D8" t="n">
-        <v>368998</v>
+        <v>104184</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>61.5%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -758,20 +758,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>359718</v>
+        <v>94904</v>
       </c>
       <c r="I8" t="n">
-        <v>24328</v>
+        <v>-5096</v>
       </c>
       <c r="J8" t="n">
-        <v>335390</v>
+        <v>100000</v>
       </c>
       <c r="K8" t="n">
-        <v>69356</v>
+        <v>29720</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>346401.9</v>
+        <v>156627.42</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>313401.9</v>
+        <v>123627.42</v>
       </c>
       <c r="I9" t="n">
-        <v>55558</v>
+        <v>-15379</v>
       </c>
       <c r="J9" t="n">
-        <v>234431</v>
+        <v>115594</v>
       </c>
       <c r="K9" t="n">
-        <v>35035</v>
+        <v>24145</v>
       </c>
     </row>
     <row r="10">
@@ -832,32 +832,32 @@
         <v>1100000</v>
       </c>
       <c r="D10" t="n">
-        <v>98784.10999999999</v>
+        <v>181559.11</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>129788</v>
+        <v>206844</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>131.4%</t>
+          <t>113.9%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>-31003.89000000001</v>
+        <v>-25284.88999999998</v>
       </c>
       <c r="I10" t="n">
-        <v>-68614</v>
+        <v>-69237</v>
       </c>
       <c r="J10" t="n">
-        <v>25401</v>
+        <v>31405</v>
       </c>
       <c r="K10" t="n">
-        <v>-25381</v>
+        <v>-5294</v>
       </c>
     </row>
     <row r="11">
@@ -875,11 +875,11 @@
         <v>400000</v>
       </c>
       <c r="D11" t="n">
-        <v>62033.8</v>
+        <v>29295.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>7.3%</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -887,20 +887,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>54912.47</v>
+        <v>22174.47</v>
       </c>
       <c r="I11" t="n">
-        <v>-4960</v>
+        <v>-5424</v>
       </c>
       <c r="J11" t="n">
-        <v>59872</v>
+        <v>27598</v>
       </c>
       <c r="K11" t="n">
-        <v>10217</v>
+        <v>8471</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>500000</v>
       </c>
       <c r="D12" t="n">
-        <v>260642</v>
+        <v>30407</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>52.1%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>52.1%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>244804</v>
+        <v>14569</v>
       </c>
       <c r="I12" t="n">
-        <v>55014</v>
+        <v>2369</v>
       </c>
       <c r="J12" t="n">
-        <v>189790</v>
+        <v>12200</v>
       </c>
       <c r="K12" t="n">
-        <v>91438</v>
+        <v>-19</v>
       </c>
     </row>
     <row r="13">
@@ -961,32 +961,32 @@
         <v>1900000</v>
       </c>
       <c r="D13" t="n">
-        <v>151554.8</v>
+        <v>104245.8</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>5.5%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>11194</v>
+        <v>244098</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>234.2%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>140360.8</v>
+        <v>-139852.2</v>
       </c>
       <c r="I13" t="n">
-        <v>15220</v>
+        <v>-174991</v>
       </c>
       <c r="J13" t="n">
-        <v>94222</v>
+        <v>4220</v>
       </c>
       <c r="K13" t="n">
-        <v>47912</v>
+        <v>-119526</v>
       </c>
     </row>
     <row r="14">
@@ -1004,11 +1004,11 @@
         <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>869279.14</v>
+        <v>226086.63</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>86.9%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1016,20 +1016,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>765631.55</v>
+        <v>122439.04</v>
       </c>
       <c r="I14" t="n">
-        <v>109381</v>
+        <v>-14588</v>
       </c>
       <c r="J14" t="n">
-        <v>634749</v>
+        <v>115527</v>
       </c>
       <c r="K14" t="n">
-        <v>354371</v>
+        <v>76165</v>
       </c>
     </row>
     <row r="15">
@@ -1047,11 +1047,11 @@
         <v>900000</v>
       </c>
       <c r="D15" t="n">
-        <v>325728.48</v>
+        <v>196528.87</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1059,20 +1059,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>292100.48</v>
+        <v>162900.87</v>
       </c>
       <c r="I15" t="n">
-        <v>60743</v>
+        <v>37966</v>
       </c>
       <c r="J15" t="n">
-        <v>181078</v>
+        <v>74588</v>
       </c>
       <c r="K15" t="n">
-        <v>59824</v>
+        <v>59086</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>134047</v>
+        <v>64187</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>121685</v>
+        <v>51825</v>
       </c>
       <c r="I16" t="n">
-        <v>26849</v>
+        <v>-4525</v>
       </c>
       <c r="J16" t="n">
-        <v>94836</v>
+        <v>56350</v>
       </c>
       <c r="K16" t="n">
-        <v>26021</v>
+        <v>28437</v>
       </c>
     </row>
     <row r="17">
@@ -1176,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>29086</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1184,24 +1184,24 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>6500</v>
+        <v>24218</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>83.3%</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>-6500</v>
+        <v>4868</v>
       </c>
       <c r="I18" t="n">
-        <v>-6500</v>
+        <v>5068</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>-200</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>12368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新看板 10月19日 — KPI685.5万(39.9%) 净流水546.3万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>224627</v>
+        <v>559077.01</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>38.6%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>80794.45</v>
+        <v>80823.45</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>143832.55</v>
+        <v>478253.56</v>
       </c>
       <c r="I2" t="n">
-        <v>145975</v>
+        <v>453051</v>
       </c>
       <c r="J2" t="n">
-        <v>-2143</v>
+        <v>25201</v>
       </c>
       <c r="K2" t="n">
-        <v>154446</v>
+        <v>430883</v>
       </c>
     </row>
     <row r="3">
@@ -531,11 +531,11 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>102457.42</v>
+        <v>240170.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -543,20 +543,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>178.6%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-80494.65000000001</v>
+        <v>57218.33999999997</v>
       </c>
       <c r="I3" t="n">
-        <v>-97792</v>
+        <v>39302</v>
       </c>
       <c r="J3" t="n">
-        <v>17297</v>
+        <v>17915</v>
       </c>
       <c r="K3" t="n">
-        <v>-62592</v>
+        <v>74324</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>272865</v>
+        <v>657617.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>47.0%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>110888.97</v>
+        <v>110926.97</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>161976.03</v>
+        <v>546690.91</v>
       </c>
       <c r="I4" t="n">
-        <v>161938</v>
+        <v>546633</v>
       </c>
       <c r="J4" t="n">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="K4" t="n">
-        <v>118982</v>
+        <v>393086</v>
       </c>
     </row>
     <row r="5">
@@ -617,11 +617,11 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>799874</v>
+        <v>1291095.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>80.7%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -629,20 +629,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>32.8%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>537315.46</v>
+        <v>1028536.82</v>
       </c>
       <c r="I5" t="n">
-        <v>393979</v>
+        <v>830200</v>
       </c>
       <c r="J5" t="n">
-        <v>143336</v>
+        <v>198336</v>
       </c>
       <c r="K5" t="n">
-        <v>503795</v>
+        <v>780206</v>
       </c>
     </row>
     <row r="6">
@@ -660,11 +660,11 @@
         <v>2500000</v>
       </c>
       <c r="D6" t="n">
-        <v>966033.92</v>
+        <v>1013467.92</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>38.6%</t>
+          <t>40.5%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -672,20 +672,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>907214.92</v>
+        <v>954648.92</v>
       </c>
       <c r="I6" t="n">
-        <v>337218</v>
+        <v>367654</v>
       </c>
       <c r="J6" t="n">
-        <v>569996</v>
+        <v>586994</v>
       </c>
       <c r="K6" t="n">
-        <v>908816</v>
+        <v>915454</v>
       </c>
     </row>
     <row r="7">
@@ -703,11 +703,11 @@
         <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>14276</v>
+        <v>93303.84</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -715,20 +715,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>38.2%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>8819</v>
+        <v>87846.84</v>
       </c>
       <c r="I7" t="n">
-        <v>11939</v>
+        <v>68365</v>
       </c>
       <c r="J7" t="n">
-        <v>-3320</v>
+        <v>19281</v>
       </c>
       <c r="K7" t="n">
-        <v>2427</v>
+        <v>21276</v>
       </c>
     </row>
     <row r="8">
@@ -746,11 +746,11 @@
         <v>600000</v>
       </c>
       <c r="D8" t="n">
-        <v>104184</v>
+        <v>382596</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>63.8%</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -758,20 +758,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>94904</v>
+        <v>373316</v>
       </c>
       <c r="I8" t="n">
-        <v>-5096</v>
+        <v>24726</v>
       </c>
       <c r="J8" t="n">
-        <v>100000</v>
+        <v>348590</v>
       </c>
       <c r="K8" t="n">
-        <v>29720</v>
+        <v>82556</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>156627.42</v>
+        <v>369595.9</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>123627.42</v>
+        <v>336595.9</v>
       </c>
       <c r="I9" t="n">
-        <v>-15379</v>
+        <v>55558</v>
       </c>
       <c r="J9" t="n">
-        <v>115594</v>
+        <v>257625</v>
       </c>
       <c r="K9" t="n">
-        <v>24145</v>
+        <v>35035</v>
       </c>
     </row>
     <row r="10">
@@ -832,11 +832,11 @@
         <v>1100000</v>
       </c>
       <c r="D10" t="n">
-        <v>181559.11</v>
+        <v>242704.11</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -844,20 +844,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>113.9%</t>
+          <t>85.2%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>-25284.88999999998</v>
+        <v>35860.11000000002</v>
       </c>
       <c r="I10" t="n">
-        <v>-69237</v>
+        <v>-63078</v>
       </c>
       <c r="J10" t="n">
-        <v>31405</v>
+        <v>86391</v>
       </c>
       <c r="K10" t="n">
-        <v>-5294</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11">
@@ -875,11 +875,11 @@
         <v>400000</v>
       </c>
       <c r="D11" t="n">
-        <v>29295.8</v>
+        <v>63761.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>7.3%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -887,20 +887,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>22174.47</v>
+        <v>56640.47</v>
       </c>
       <c r="I11" t="n">
-        <v>-5424</v>
+        <v>-4912</v>
       </c>
       <c r="J11" t="n">
-        <v>27598</v>
+        <v>61552</v>
       </c>
       <c r="K11" t="n">
-        <v>8471</v>
+        <v>11945</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>500000</v>
       </c>
       <c r="D12" t="n">
-        <v>30407</v>
+        <v>261438</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>52.3%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>52.1%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>14569</v>
+        <v>245600</v>
       </c>
       <c r="I12" t="n">
-        <v>2369</v>
+        <v>55810</v>
       </c>
       <c r="J12" t="n">
-        <v>12200</v>
+        <v>189790</v>
       </c>
       <c r="K12" t="n">
-        <v>-19</v>
+        <v>91438</v>
       </c>
     </row>
     <row r="13">
@@ -961,11 +961,11 @@
         <v>1900000</v>
       </c>
       <c r="D13" t="n">
-        <v>104245.8</v>
+        <v>210874.8</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -973,20 +973,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>234.2%</t>
+          <t>115.8%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-139852.2</v>
+        <v>-33223.20000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>-174991</v>
+        <v>-160990</v>
       </c>
       <c r="J13" t="n">
-        <v>4220</v>
+        <v>96848</v>
       </c>
       <c r="K13" t="n">
-        <v>-119526</v>
+        <v>-101357</v>
       </c>
     </row>
     <row r="14">
@@ -1004,11 +1004,11 @@
         <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>226086.63</v>
+        <v>920064.14</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>92.0%</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1016,20 +1016,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>122439.04</v>
+        <v>816416.55</v>
       </c>
       <c r="I14" t="n">
-        <v>-14588</v>
+        <v>129270</v>
       </c>
       <c r="J14" t="n">
-        <v>115527</v>
+        <v>665645</v>
       </c>
       <c r="K14" t="n">
-        <v>76165</v>
+        <v>382370</v>
       </c>
     </row>
     <row r="15">
@@ -1047,11 +1047,11 @@
         <v>900000</v>
       </c>
       <c r="D15" t="n">
-        <v>196528.87</v>
+        <v>372511.87</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>41.4%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1059,20 +1059,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>162900.87</v>
+        <v>338883.87</v>
       </c>
       <c r="I15" t="n">
-        <v>37966</v>
+        <v>89561</v>
       </c>
       <c r="J15" t="n">
-        <v>74588</v>
+        <v>198976</v>
       </c>
       <c r="K15" t="n">
-        <v>59086</v>
+        <v>59891</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>64187</v>
+        <v>147693</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>51825</v>
+        <v>135331</v>
       </c>
       <c r="I16" t="n">
-        <v>-4525</v>
+        <v>26878</v>
       </c>
       <c r="J16" t="n">
-        <v>56350</v>
+        <v>108453</v>
       </c>
       <c r="K16" t="n">
-        <v>28437</v>
+        <v>39269</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
更新看板 10月20日 — KPI692.5万(40.3%) 净流水536.6万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>559077.01</v>
+        <v>564019.01</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>38.6%</t>
+          <t>38.9%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>80823.45</v>
+        <v>97723.45</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>478253.56</v>
+        <v>466295.56</v>
       </c>
       <c r="I2" t="n">
-        <v>453051</v>
+        <v>441093</v>
       </c>
       <c r="J2" t="n">
         <v>25201</v>
       </c>
       <c r="K2" t="n">
-        <v>430883</v>
+        <v>418925</v>
       </c>
     </row>
     <row r="3">
@@ -539,24 +539,24 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>182952.07</v>
+        <v>188021.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>76.2%</t>
+          <t>78.3%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>57218.33999999997</v>
+        <v>52149.34</v>
       </c>
       <c r="I3" t="n">
-        <v>39302</v>
+        <v>34233</v>
       </c>
       <c r="J3" t="n">
         <v>17915</v>
       </c>
       <c r="K3" t="n">
-        <v>74324</v>
+        <v>69255</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>657617.88</v>
+        <v>667558.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>47.7%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>110926.97</v>
+        <v>149341.97</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>546690.91</v>
+        <v>518216.91</v>
       </c>
       <c r="I4" t="n">
-        <v>546633</v>
+        <v>518159</v>
       </c>
       <c r="J4" t="n">
         <v>57</v>
       </c>
       <c r="K4" t="n">
-        <v>393086</v>
+        <v>396810</v>
       </c>
     </row>
     <row r="5">
@@ -617,32 +617,32 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1291095.36</v>
+        <v>1261983.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>78.9%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>262558.54</v>
+        <v>299119.54</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>23.7%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1028536.82</v>
+        <v>962863.8199999998</v>
       </c>
       <c r="I5" t="n">
-        <v>830200</v>
+        <v>750539</v>
       </c>
       <c r="J5" t="n">
-        <v>198336</v>
+        <v>212324</v>
       </c>
       <c r="K5" t="n">
-        <v>780206</v>
+        <v>760333</v>
       </c>
     </row>
     <row r="6">
@@ -660,11 +660,11 @@
         <v>2500000</v>
       </c>
       <c r="D6" t="n">
-        <v>1013467.92</v>
+        <v>1041378.92</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>40.5%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -672,20 +672,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>954648.92</v>
+        <v>982559.92</v>
       </c>
       <c r="I6" t="n">
-        <v>367654</v>
+        <v>382386</v>
       </c>
       <c r="J6" t="n">
-        <v>586994</v>
+        <v>600173</v>
       </c>
       <c r="K6" t="n">
-        <v>915454</v>
+        <v>943365</v>
       </c>
     </row>
     <row r="7">
@@ -703,32 +703,32 @@
         <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>93303.84</v>
+        <v>91623.84</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5457</v>
+        <v>7857</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>87846.84</v>
+        <v>83766.84</v>
       </c>
       <c r="I7" t="n">
-        <v>68365</v>
+        <v>65965</v>
       </c>
       <c r="J7" t="n">
-        <v>19281</v>
+        <v>17601</v>
       </c>
       <c r="K7" t="n">
-        <v>21276</v>
+        <v>19596</v>
       </c>
     </row>
     <row r="8">
@@ -789,7 +789,7 @@
         <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>369595.9</v>
+        <v>370371.98</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -797,24 +797,24 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>33000</v>
+        <v>36519</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>336595.9</v>
+        <v>333852.98</v>
       </c>
       <c r="I9" t="n">
-        <v>55558</v>
+        <v>52039</v>
       </c>
       <c r="J9" t="n">
         <v>257625</v>
       </c>
       <c r="K9" t="n">
-        <v>35035</v>
+        <v>35792</v>
       </c>
     </row>
     <row r="10">
@@ -832,11 +832,11 @@
         <v>1100000</v>
       </c>
       <c r="D10" t="n">
-        <v>242704.11</v>
+        <v>206497.87</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -844,20 +844,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>85.2%</t>
+          <t>100.2%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>35860.11000000002</v>
+        <v>-346.1300000000047</v>
       </c>
       <c r="I10" t="n">
-        <v>-63078</v>
+        <v>-63505</v>
       </c>
       <c r="J10" t="n">
-        <v>86391</v>
+        <v>49393</v>
       </c>
       <c r="K10" t="n">
-        <v>266</v>
+        <v>-24944</v>
       </c>
     </row>
     <row r="11">
@@ -875,7 +875,7 @@
         <v>400000</v>
       </c>
       <c r="D11" t="n">
-        <v>63761.8</v>
+        <v>63608</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -883,24 +883,24 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>7121.33</v>
+        <v>29921.33</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>47.0%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>56640.47</v>
+        <v>33686.67</v>
       </c>
       <c r="I11" t="n">
-        <v>-4912</v>
+        <v>-4941</v>
       </c>
       <c r="J11" t="n">
-        <v>61552</v>
+        <v>38628</v>
       </c>
       <c r="K11" t="n">
-        <v>11945</v>
+        <v>-11008</v>
       </c>
     </row>
     <row r="12">
@@ -961,32 +961,32 @@
         <v>1900000</v>
       </c>
       <c r="D13" t="n">
-        <v>210874.8</v>
+        <v>258457.4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>244098</v>
+        <v>268077</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>115.8%</t>
+          <t>103.7%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-33223.20000000001</v>
+        <v>-9619.600000000006</v>
       </c>
       <c r="I13" t="n">
-        <v>-160990</v>
+        <v>-135657</v>
       </c>
       <c r="J13" t="n">
-        <v>96848</v>
+        <v>94868</v>
       </c>
       <c r="K13" t="n">
-        <v>-101357</v>
+        <v>-77753</v>
       </c>
     </row>
     <row r="14">
@@ -1004,7 +1004,7 @@
         <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>920064.14</v>
+        <v>920064.1400000001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1012,24 +1012,24 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>103647.59</v>
+        <v>110247.59</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>816416.55</v>
+        <v>809816.5500000002</v>
       </c>
       <c r="I14" t="n">
-        <v>129270</v>
+        <v>122272</v>
       </c>
       <c r="J14" t="n">
-        <v>665645</v>
+        <v>666043</v>
       </c>
       <c r="K14" t="n">
-        <v>382370</v>
+        <v>375770</v>
       </c>
     </row>
     <row r="15">
@@ -1047,32 +1047,32 @@
         <v>900000</v>
       </c>
       <c r="D15" t="n">
-        <v>372511.87</v>
+        <v>373364.21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>41.4%</t>
+          <t>41.5%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>33628</v>
+        <v>38128</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>338883.87</v>
+        <v>335236.21</v>
       </c>
       <c r="I15" t="n">
-        <v>89561</v>
+        <v>89163</v>
       </c>
       <c r="J15" t="n">
-        <v>198976</v>
+        <v>194874</v>
       </c>
       <c r="K15" t="n">
-        <v>59891</v>
+        <v>60744</v>
       </c>
     </row>
     <row r="16">
@@ -1098,24 +1098,24 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>12362</v>
+        <v>17381</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>135331</v>
+        <v>130312</v>
       </c>
       <c r="I16" t="n">
-        <v>26878</v>
+        <v>26859</v>
       </c>
       <c r="J16" t="n">
-        <v>108453</v>
+        <v>103453</v>
       </c>
       <c r="K16" t="n">
-        <v>39269</v>
+        <v>39250</v>
       </c>
     </row>
     <row r="17">
@@ -1176,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>29086</v>
+        <v>74457</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1184,24 +1184,24 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>24218</v>
+        <v>26217</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>35.2%</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>4868</v>
+        <v>48240</v>
       </c>
       <c r="I18" t="n">
-        <v>5068</v>
+        <v>48440</v>
       </c>
       <c r="J18" t="n">
         <v>-200</v>
       </c>
       <c r="K18" t="n">
-        <v>12368</v>
+        <v>55740</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新看板 10月21日 — KPI975.0万(56.7%) 净流水793.7万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>564019.01</v>
+        <v>651711.3100000001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>38.9%</t>
+          <t>44.9%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>97723.45</v>
+        <v>121033.45</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>466295.56</v>
+        <v>530677.8600000001</v>
       </c>
       <c r="I2" t="n">
-        <v>441093</v>
+        <v>499174</v>
       </c>
       <c r="J2" t="n">
-        <v>25201</v>
+        <v>31502</v>
       </c>
       <c r="K2" t="n">
-        <v>418925</v>
+        <v>469011</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>240170.41</v>
+        <v>282567.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>188021.07</v>
+        <v>220151.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>78.3%</t>
+          <t>77.9%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>52149.34</v>
+        <v>62416.33999999997</v>
       </c>
       <c r="I3" t="n">
-        <v>34233</v>
+        <v>43000</v>
       </c>
       <c r="J3" t="n">
-        <v>17915</v>
+        <v>19415</v>
       </c>
       <c r="K3" t="n">
-        <v>69255</v>
+        <v>76122</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>667558.88</v>
+        <v>747913.78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>47.7%</t>
+          <t>53.4%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>149341.97</v>
+        <v>158534.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>518216.91</v>
+        <v>589378.91</v>
       </c>
       <c r="I4" t="n">
-        <v>518159</v>
+        <v>589321</v>
       </c>
       <c r="J4" t="n">
         <v>57</v>
       </c>
       <c r="K4" t="n">
-        <v>396810</v>
+        <v>456608</v>
       </c>
     </row>
     <row r="5">
@@ -617,32 +617,32 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1261983.36</v>
+        <v>1394627.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>78.9%</t>
+          <t>87.2%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>299119.54</v>
+        <v>349147.54</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>962863.8199999998</v>
+        <v>1045479.82</v>
       </c>
       <c r="I5" t="n">
-        <v>750539</v>
+        <v>834656</v>
       </c>
       <c r="J5" t="n">
-        <v>212324</v>
+        <v>210823</v>
       </c>
       <c r="K5" t="n">
-        <v>760333</v>
+        <v>810251</v>
       </c>
     </row>
     <row r="6">
@@ -660,32 +660,32 @@
         <v>2500000</v>
       </c>
       <c r="D6" t="n">
-        <v>1041378.92</v>
+        <v>1134208.92</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>45.4%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>58819</v>
+        <v>60819</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>5.4%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>982559.92</v>
+        <v>1073389.92</v>
       </c>
       <c r="I6" t="n">
-        <v>382386</v>
+        <v>28987</v>
       </c>
       <c r="J6" t="n">
-        <v>600173</v>
+        <v>1044402</v>
       </c>
       <c r="K6" t="n">
-        <v>943365</v>
+        <v>1035797</v>
       </c>
     </row>
     <row r="7">
@@ -703,11 +703,11 @@
         <v>500000</v>
       </c>
       <c r="D7" t="n">
-        <v>91623.84</v>
+        <v>139415.84</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -715,20 +715,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>83766.84</v>
+        <v>131558.84</v>
       </c>
       <c r="I7" t="n">
-        <v>65965</v>
+        <v>79159</v>
       </c>
       <c r="J7" t="n">
-        <v>17601</v>
+        <v>51999</v>
       </c>
       <c r="K7" t="n">
-        <v>19596</v>
+        <v>19796</v>
       </c>
     </row>
     <row r="8">
@@ -746,32 +746,32 @@
         <v>600000</v>
       </c>
       <c r="D8" t="n">
-        <v>382596</v>
+        <v>405687</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>67.6%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>9280</v>
+        <v>11280</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>2.8%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>373316</v>
+        <v>394407</v>
       </c>
       <c r="I8" t="n">
-        <v>24726</v>
+        <v>25423</v>
       </c>
       <c r="J8" t="n">
-        <v>348590</v>
+        <v>368984</v>
       </c>
       <c r="K8" t="n">
-        <v>82556</v>
+        <v>84049</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>1000000</v>
       </c>
       <c r="D9" t="n">
-        <v>370371.98</v>
+        <v>441271.58</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>37.0%</t>
+          <t>44.1%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>333852.98</v>
+        <v>404752.58</v>
       </c>
       <c r="I9" t="n">
-        <v>52039</v>
+        <v>43589</v>
       </c>
       <c r="J9" t="n">
-        <v>257625</v>
+        <v>335638</v>
       </c>
       <c r="K9" t="n">
-        <v>35792</v>
+        <v>37504</v>
       </c>
     </row>
     <row r="10">
@@ -832,32 +832,32 @@
         <v>1100000</v>
       </c>
       <c r="D10" t="n">
-        <v>206497.87</v>
+        <v>687024.87</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>206844</v>
+        <v>259842</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>100.2%</t>
+          <t>37.8%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>-346.1300000000047</v>
+        <v>427182.87</v>
       </c>
       <c r="I10" t="n">
-        <v>-63505</v>
+        <v>114773</v>
       </c>
       <c r="J10" t="n">
-        <v>49393</v>
+        <v>298644</v>
       </c>
       <c r="K10" t="n">
-        <v>-24944</v>
+        <v>342608</v>
       </c>
     </row>
     <row r="11">
@@ -875,32 +875,32 @@
         <v>400000</v>
       </c>
       <c r="D11" t="n">
-        <v>63608</v>
+        <v>71780.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>29921.33</v>
+        <v>41921.33</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>58.4%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>33686.67</v>
+        <v>29859.47</v>
       </c>
       <c r="I11" t="n">
-        <v>-4941</v>
+        <v>-4893</v>
       </c>
       <c r="J11" t="n">
-        <v>38628</v>
+        <v>34752</v>
       </c>
       <c r="K11" t="n">
-        <v>-11008</v>
+        <v>-10835</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>500000</v>
       </c>
       <c r="D12" t="n">
-        <v>261438</v>
+        <v>262957</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>52.3%</t>
+          <t>52.6%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>245600</v>
+        <v>247119</v>
       </c>
       <c r="I12" t="n">
-        <v>55810</v>
+        <v>55829</v>
       </c>
       <c r="J12" t="n">
-        <v>189790</v>
+        <v>191290</v>
       </c>
       <c r="K12" t="n">
-        <v>91438</v>
+        <v>91457</v>
       </c>
     </row>
     <row r="13">
@@ -961,32 +961,32 @@
         <v>1900000</v>
       </c>
       <c r="D13" t="n">
-        <v>258457.4</v>
+        <v>1463526.4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>268077</v>
+        <v>285476</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>103.7%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-9619.600000000006</v>
+        <v>1178050.4</v>
       </c>
       <c r="I13" t="n">
-        <v>-135657</v>
+        <v>1015013</v>
       </c>
       <c r="J13" t="n">
-        <v>94868</v>
+        <v>131868</v>
       </c>
       <c r="K13" t="n">
-        <v>-77753</v>
+        <v>1083418</v>
       </c>
     </row>
     <row r="14">
@@ -1004,11 +1004,11 @@
         <v>1000000</v>
       </c>
       <c r="D14" t="n">
-        <v>920064.1400000001</v>
+        <v>938917.14</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>93.9%</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1016,20 +1016,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>11.7%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>809816.5500000002</v>
+        <v>828669.55</v>
       </c>
       <c r="I14" t="n">
-        <v>122272</v>
+        <v>126849</v>
       </c>
       <c r="J14" t="n">
-        <v>666043</v>
+        <v>680319</v>
       </c>
       <c r="K14" t="n">
-        <v>375770</v>
+        <v>382229</v>
       </c>
     </row>
     <row r="15">
@@ -1047,11 +1047,11 @@
         <v>900000</v>
       </c>
       <c r="D15" t="n">
-        <v>373364.21</v>
+        <v>387112.21</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>41.5%</t>
+          <t>43.0%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1059,20 +1059,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>335236.21</v>
+        <v>348984.21</v>
       </c>
       <c r="I15" t="n">
-        <v>89163</v>
+        <v>89211</v>
       </c>
       <c r="J15" t="n">
-        <v>194874</v>
+        <v>208574</v>
       </c>
       <c r="K15" t="n">
-        <v>60744</v>
+        <v>60792</v>
       </c>
     </row>
     <row r="16">
@@ -1090,32 +1090,32 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>147693</v>
+        <v>170797</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>17381</v>
+        <v>38831</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>130312</v>
+        <v>131966</v>
       </c>
       <c r="I16" t="n">
-        <v>26859</v>
+        <v>26868</v>
       </c>
       <c r="J16" t="n">
-        <v>103453</v>
+        <v>105098</v>
       </c>
       <c r="K16" t="n">
-        <v>39250</v>
+        <v>39558</v>
       </c>
     </row>
     <row r="17">
@@ -1176,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>74457</v>
+        <v>570839.8</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1184,24 +1184,24 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>26217</v>
+        <v>58137</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>35.2%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>48240</v>
+        <v>512702.8</v>
       </c>
       <c r="I18" t="n">
-        <v>48440</v>
+        <v>512521</v>
       </c>
       <c r="J18" t="n">
-        <v>-200</v>
+        <v>181</v>
       </c>
       <c r="K18" t="n">
-        <v>55740</v>
+        <v>484406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
更新看板 10月24日 — KPI1173.8万(63.4%) 净流水973.2万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -429,12 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>目标</t>
+          <t>目标(元)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>完成</t>
+          <t>完成(元)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>本月退费</t>
+          <t>本月退费(元)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -454,22 +454,22 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>本月净流水</t>
+          <t>本月净流水(元)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>新客净流水</t>
+          <t>新客净流水(元)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>老客净流水</t>
+          <t>老客净流水(元)</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>非1V1及菌群净</t>
+          <t>非1V1及菌群净(元)</t>
         </is>
       </c>
     </row>
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>783326.16</v>
+        <v>881795.39</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>60.8%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>129547.45</v>
+        <v>134561.15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>653778.7100000001</v>
+        <v>747234.24</v>
       </c>
       <c r="I2" t="n">
-        <v>621580</v>
+        <v>714980</v>
       </c>
       <c r="J2" t="n">
-        <v>32198</v>
+        <v>32253</v>
       </c>
       <c r="K2" t="n">
-        <v>591514</v>
+        <v>684174</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>325870.41</v>
+        <v>383448.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>220402.07</v>
+        <v>250667.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>67.6%</t>
+          <t>65.4%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>105468.34</v>
+        <v>132781.34</v>
       </c>
       <c r="I3" t="n">
-        <v>86052</v>
+        <v>93565</v>
       </c>
       <c r="J3" t="n">
-        <v>19415</v>
+        <v>39215</v>
       </c>
       <c r="K3" t="n">
-        <v>119174</v>
+        <v>146487</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>824725.78</v>
+        <v>920969.78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>58.9%</t>
+          <t>65.8%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>162922.87</v>
+        <v>167221.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>661802.91</v>
+        <v>753747.91</v>
       </c>
       <c r="I4" t="n">
-        <v>665522</v>
+        <v>757467</v>
       </c>
       <c r="J4" t="n">
         <v>-3720</v>
       </c>
       <c r="K4" t="n">
-        <v>507032</v>
+        <v>564565</v>
       </c>
     </row>
     <row r="5">
@@ -617,11 +617,11 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1446274.36</v>
+        <v>1506000.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>90.4%</t>
+          <t>94.1%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -629,20 +629,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1087126.82</v>
+        <v>1146852.82</v>
       </c>
       <c r="I5" t="n">
-        <v>876303</v>
+        <v>924029</v>
       </c>
       <c r="J5" t="n">
-        <v>210823</v>
+        <v>222823</v>
       </c>
       <c r="K5" t="n">
-        <v>837078</v>
+        <v>884206</v>
       </c>
     </row>
     <row r="6">
@@ -660,11 +660,11 @@
         <v>1300000</v>
       </c>
       <c r="D6" t="n">
-        <v>588664</v>
+        <v>549614</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>45.3%</t>
+          <t>42.3%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -672,20 +672,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>543904</v>
+        <v>504854</v>
       </c>
       <c r="I6" t="n">
-        <v>542824</v>
+        <v>503774</v>
       </c>
       <c r="J6" t="n">
         <v>1080</v>
       </c>
       <c r="K6" t="n">
-        <v>484910</v>
+        <v>445860</v>
       </c>
     </row>
     <row r="7">
@@ -703,32 +703,32 @@
         <v>2500000</v>
       </c>
       <c r="D7" t="n">
-        <v>1184871</v>
+        <v>1419809.8</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>47.4%</t>
+          <t>56.8%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>60819</v>
+        <v>65819</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1124052</v>
+        <v>1353990.8</v>
       </c>
       <c r="I7" t="n">
-        <v>428226</v>
+        <v>560491</v>
       </c>
       <c r="J7" t="n">
-        <v>695826</v>
+        <v>793499</v>
       </c>
       <c r="K7" t="n">
-        <v>1086460</v>
+        <v>1319800</v>
       </c>
     </row>
     <row r="8">
@@ -746,32 +746,32 @@
         <v>500000</v>
       </c>
       <c r="D8" t="n">
-        <v>153032.84</v>
+        <v>178081.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>30.6%</t>
+          <t>35.6%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7857</v>
+        <v>15857</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>145175.84</v>
+        <v>162224.84</v>
       </c>
       <c r="I8" t="n">
-        <v>92776</v>
+        <v>106431</v>
       </c>
       <c r="J8" t="n">
-        <v>51999</v>
+        <v>55393</v>
       </c>
       <c r="K8" t="n">
-        <v>33015</v>
+        <v>46272</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>600000</v>
       </c>
       <c r="D9" t="n">
-        <v>413102</v>
+        <v>439088</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>68.9%</t>
+          <t>73.2%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.7%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>401822</v>
+        <v>427808</v>
       </c>
       <c r="I9" t="n">
-        <v>25044</v>
+        <v>25442</v>
       </c>
       <c r="J9" t="n">
-        <v>376778</v>
+        <v>402366</v>
       </c>
       <c r="K9" t="n">
-        <v>91066</v>
+        <v>106654</v>
       </c>
     </row>
     <row r="10">
@@ -832,32 +832,32 @@
         <v>1000000</v>
       </c>
       <c r="D10" t="n">
-        <v>471427.33</v>
+        <v>501128.33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>47.1%</t>
+          <t>50.1%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>36519</v>
+        <v>53319</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>434908.33</v>
+        <v>447809.33</v>
       </c>
       <c r="I10" t="n">
-        <v>43646</v>
+        <v>43884</v>
       </c>
       <c r="J10" t="n">
-        <v>365638</v>
+        <v>376736</v>
       </c>
       <c r="K10" t="n">
-        <v>37660</v>
+        <v>22663</v>
       </c>
     </row>
     <row r="11">
@@ -875,32 +875,32 @@
         <v>1100000</v>
       </c>
       <c r="D11" t="n">
-        <v>684757.87</v>
+        <v>705956.27</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>62.3%</t>
+          <t>64.2%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>265441</v>
+        <v>265839</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>37.7%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>419316.87</v>
+        <v>440117.27</v>
       </c>
       <c r="I11" t="n">
-        <v>110109</v>
+        <v>115663</v>
       </c>
       <c r="J11" t="n">
-        <v>295442</v>
+        <v>309234</v>
       </c>
       <c r="K11" t="n">
-        <v>337148</v>
+        <v>343359</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>400000</v>
       </c>
       <c r="D12" t="n">
-        <v>80605.8</v>
+        <v>108424.8</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>27.1%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>38.7%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>38655.47</v>
+        <v>66474.47</v>
       </c>
       <c r="I12" t="n">
-        <v>-4495</v>
+        <v>-4476</v>
       </c>
       <c r="J12" t="n">
-        <v>43150</v>
+        <v>70950</v>
       </c>
       <c r="K12" t="n">
-        <v>-10835</v>
+        <v>8983</v>
       </c>
     </row>
     <row r="13">
@@ -961,32 +961,32 @@
         <v>500000</v>
       </c>
       <c r="D13" t="n">
-        <v>262957</v>
+        <v>263772</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>52.6%</t>
+          <t>52.8%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>15838</v>
+        <v>45638</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>247119</v>
+        <v>218134</v>
       </c>
       <c r="I13" t="n">
-        <v>55829</v>
+        <v>56246</v>
       </c>
       <c r="J13" t="n">
-        <v>191290</v>
+        <v>161888</v>
       </c>
       <c r="K13" t="n">
-        <v>91457</v>
+        <v>61676</v>
       </c>
     </row>
     <row r="14">
@@ -1004,32 +1004,32 @@
         <v>1900000</v>
       </c>
       <c r="D14" t="n">
-        <v>1465620.4</v>
+        <v>1880717.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>77.1%</t>
+          <t>99.0%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>305912</v>
+        <v>314950</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1159708.4</v>
+        <v>1565767.1</v>
       </c>
       <c r="I14" t="n">
-        <v>1016671</v>
+        <v>1295876</v>
       </c>
       <c r="J14" t="n">
-        <v>111868</v>
+        <v>236922</v>
       </c>
       <c r="K14" t="n">
-        <v>1085474</v>
+        <v>1392123</v>
       </c>
     </row>
     <row r="15">
@@ -1047,32 +1047,32 @@
         <v>1000000</v>
       </c>
       <c r="D15" t="n">
-        <v>966916.14</v>
+        <v>1165591.04</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>96.7%</t>
+          <t>116.6%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>114266.59</v>
+        <v>115766.59</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>852649.55</v>
+        <v>1049824.45</v>
       </c>
       <c r="I15" t="n">
-        <v>126849</v>
+        <v>180724</v>
       </c>
       <c r="J15" t="n">
-        <v>704299</v>
+        <v>847599</v>
       </c>
       <c r="K15" t="n">
-        <v>384209</v>
+        <v>443370</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>408765.21</v>
+        <v>556070.89</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>45.4%</t>
+          <t>61.8%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>341818.21</v>
+        <v>489123.89</v>
       </c>
       <c r="I16" t="n">
-        <v>97128</v>
+        <v>124122</v>
       </c>
       <c r="J16" t="n">
-        <v>193491</v>
+        <v>312889</v>
       </c>
       <c r="K16" t="n">
-        <v>36030</v>
+        <v>62743</v>
       </c>
     </row>
     <row r="17">
@@ -1133,11 +1133,11 @@
         <v>900000</v>
       </c>
       <c r="D17" t="n">
-        <v>183273</v>
+        <v>244358</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>27.2%</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1145,20 +1145,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>144423</v>
+        <v>205508</v>
       </c>
       <c r="I17" t="n">
-        <v>26849</v>
+        <v>47934</v>
       </c>
       <c r="J17" t="n">
-        <v>117574</v>
+        <v>157574</v>
       </c>
       <c r="K17" t="n">
-        <v>41219</v>
+        <v>42304</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
更新看板 10月25日 — KPI1243.1万(67.2%) 净流水1042.4万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>881795.39</v>
+        <v>919807.3899999999</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>60.8%</t>
+          <t>63.4%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>134561.15</v>
+        <v>134760.15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>747234.24</v>
+        <v>785047.2399999999</v>
       </c>
       <c r="I2" t="n">
-        <v>714980</v>
+        <v>752774</v>
       </c>
       <c r="J2" t="n">
-        <v>32253</v>
+        <v>32272</v>
       </c>
       <c r="K2" t="n">
-        <v>684174</v>
+        <v>721589</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>383448.41</v>
+        <v>385575.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>250667.07</v>
+        <v>250956.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>65.4%</t>
+          <t>65.1%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>132781.34</v>
+        <v>134619.34</v>
       </c>
       <c r="I3" t="n">
-        <v>93565</v>
+        <v>95403</v>
       </c>
       <c r="J3" t="n">
         <v>39215</v>
       </c>
       <c r="K3" t="n">
-        <v>146487</v>
+        <v>147927</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>920969.78</v>
+        <v>964120.78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>65.8%</t>
+          <t>68.9%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>167221.87</v>
+        <v>167325.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>753747.91</v>
+        <v>796794.91</v>
       </c>
       <c r="I4" t="n">
-        <v>757467</v>
+        <v>800514</v>
       </c>
       <c r="J4" t="n">
         <v>-3720</v>
       </c>
       <c r="K4" t="n">
-        <v>564565</v>
+        <v>607612</v>
       </c>
     </row>
     <row r="5">
@@ -617,11 +617,11 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1506000.36</v>
+        <v>1536337.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>94.1%</t>
+          <t>96.0%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -629,20 +629,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1146852.82</v>
+        <v>1177189.82</v>
       </c>
       <c r="I5" t="n">
-        <v>924029</v>
+        <v>944366</v>
       </c>
       <c r="J5" t="n">
-        <v>222823</v>
+        <v>232823</v>
       </c>
       <c r="K5" t="n">
-        <v>884206</v>
+        <v>904543</v>
       </c>
     </row>
     <row r="6">
@@ -703,11 +703,11 @@
         <v>2500000</v>
       </c>
       <c r="D7" t="n">
-        <v>1419809.8</v>
+        <v>1498813.799999999</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>56.8%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -715,20 +715,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4.6%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1353990.8</v>
+        <v>1432994.799999999</v>
       </c>
       <c r="I7" t="n">
-        <v>560491</v>
+        <v>583091</v>
       </c>
       <c r="J7" t="n">
-        <v>793499</v>
+        <v>849903</v>
       </c>
       <c r="K7" t="n">
-        <v>1319800</v>
+        <v>1398804</v>
       </c>
     </row>
     <row r="8">
@@ -746,32 +746,32 @@
         <v>500000</v>
       </c>
       <c r="D8" t="n">
-        <v>178081.84</v>
+        <v>186081.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>35.6%</t>
+          <t>37.2%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>15857</v>
+        <v>15876</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>162224.84</v>
+        <v>170205.84</v>
       </c>
       <c r="I8" t="n">
-        <v>106431</v>
+        <v>106014</v>
       </c>
       <c r="J8" t="n">
-        <v>55393</v>
+        <v>63791</v>
       </c>
       <c r="K8" t="n">
-        <v>46272</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>600000</v>
       </c>
       <c r="D9" t="n">
-        <v>439088</v>
+        <v>439884</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>73.2%</t>
+          <t>73.3%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -805,13 +805,13 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>427808</v>
+        <v>428604</v>
       </c>
       <c r="I9" t="n">
-        <v>25442</v>
+        <v>25840</v>
       </c>
       <c r="J9" t="n">
-        <v>402366</v>
+        <v>402764</v>
       </c>
       <c r="K9" t="n">
         <v>106654</v>
@@ -832,11 +832,11 @@
         <v>1000000</v>
       </c>
       <c r="D10" t="n">
-        <v>501128.33</v>
+        <v>517343.33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>50.1%</t>
+          <t>51.7%</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -844,20 +844,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>447809.33</v>
+        <v>464024.33</v>
       </c>
       <c r="I10" t="n">
-        <v>43884</v>
+        <v>44501</v>
       </c>
       <c r="J10" t="n">
-        <v>376736</v>
+        <v>392334</v>
       </c>
       <c r="K10" t="n">
-        <v>22663</v>
+        <v>22882</v>
       </c>
     </row>
     <row r="11">
@@ -875,11 +875,11 @@
         <v>1100000</v>
       </c>
       <c r="D11" t="n">
-        <v>705956.27</v>
+        <v>759104.4700000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>64.2%</t>
+          <t>69.0%</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -887,20 +887,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>440117.27</v>
+        <v>493265.4700000001</v>
       </c>
       <c r="I11" t="n">
-        <v>115663</v>
+        <v>145720</v>
       </c>
       <c r="J11" t="n">
-        <v>309234</v>
+        <v>329670</v>
       </c>
       <c r="K11" t="n">
-        <v>343359</v>
+        <v>395909</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>400000</v>
       </c>
       <c r="D12" t="n">
-        <v>108424.8</v>
+        <v>125262.8</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>31.3%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>38.7%</t>
+          <t>33.5%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>66474.47</v>
+        <v>83312.47</v>
       </c>
       <c r="I12" t="n">
-        <v>-4476</v>
+        <v>-4036</v>
       </c>
       <c r="J12" t="n">
-        <v>70950</v>
+        <v>87348</v>
       </c>
       <c r="K12" t="n">
-        <v>8983</v>
+        <v>9025</v>
       </c>
     </row>
     <row r="13">
@@ -961,11 +961,11 @@
         <v>500000</v>
       </c>
       <c r="D13" t="n">
-        <v>263772</v>
+        <v>264787</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>53.0%</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -973,20 +973,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>218134</v>
+        <v>219149</v>
       </c>
       <c r="I13" t="n">
-        <v>56246</v>
+        <v>57261</v>
       </c>
       <c r="J13" t="n">
         <v>161888</v>
       </c>
       <c r="K13" t="n">
-        <v>61676</v>
+        <v>61695</v>
       </c>
     </row>
     <row r="14">
@@ -1004,32 +1004,32 @@
         <v>1900000</v>
       </c>
       <c r="D14" t="n">
-        <v>1880717.1</v>
+        <v>2080770.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>99.0%</t>
+          <t>109.5%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>314950</v>
+        <v>314959</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1565767.1</v>
+        <v>1765811.1</v>
       </c>
       <c r="I14" t="n">
-        <v>1295876</v>
+        <v>1361425</v>
       </c>
       <c r="J14" t="n">
-        <v>236922</v>
+        <v>321417</v>
       </c>
       <c r="K14" t="n">
-        <v>1392123</v>
+        <v>1489571</v>
       </c>
     </row>
     <row r="15">
@@ -1047,11 +1047,11 @@
         <v>1000000</v>
       </c>
       <c r="D15" t="n">
-        <v>1165591.04</v>
+        <v>1249760.04</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>116.6%</t>
+          <t>125.0%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1059,20 +1059,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1049824.45</v>
+        <v>1133993.45</v>
       </c>
       <c r="I15" t="n">
-        <v>180724</v>
+        <v>214715</v>
       </c>
       <c r="J15" t="n">
-        <v>847599</v>
+        <v>897777</v>
       </c>
       <c r="K15" t="n">
-        <v>443370</v>
+        <v>485045</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>556070.89</v>
+        <v>614278.62</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>68.3%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>489123.89</v>
+        <v>547331.62</v>
       </c>
       <c r="I16" t="n">
-        <v>124122</v>
+        <v>124922</v>
       </c>
       <c r="J16" t="n">
-        <v>312889</v>
+        <v>369189</v>
       </c>
       <c r="K16" t="n">
-        <v>62743</v>
+        <v>63851</v>
       </c>
     </row>
     <row r="17">
@@ -1133,11 +1133,11 @@
         <v>900000</v>
       </c>
       <c r="D17" t="n">
-        <v>244358</v>
+        <v>306373</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1145,20 +1145,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>205508</v>
+        <v>267523</v>
       </c>
       <c r="I17" t="n">
-        <v>47934</v>
+        <v>39153</v>
       </c>
       <c r="J17" t="n">
-        <v>157574</v>
+        <v>228370</v>
       </c>
       <c r="K17" t="n">
-        <v>42304</v>
+        <v>42323</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
更新看板 10月26日 — KPI1311.0万(70.9%) 净流水1099.9万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>919807.3899999999</v>
+        <v>1017174.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>70.1%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>134760.15</v>
+        <v>166896.15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>785047.2399999999</v>
+        <v>850278.2499999999</v>
       </c>
       <c r="I2" t="n">
-        <v>752774</v>
+        <v>818005</v>
       </c>
       <c r="J2" t="n">
         <v>32272</v>
       </c>
       <c r="K2" t="n">
-        <v>721589</v>
+        <v>805426</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>385575.41</v>
+        <v>442206.41</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>30.5%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>250956.07</v>
+        <v>251409.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>65.1%</t>
+          <t>56.9%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>134619.34</v>
+        <v>190797.34</v>
       </c>
       <c r="I3" t="n">
-        <v>95403</v>
+        <v>151562</v>
       </c>
       <c r="J3" t="n">
-        <v>39215</v>
+        <v>39234</v>
       </c>
       <c r="K3" t="n">
-        <v>147927</v>
+        <v>203707</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>964120.78</v>
+        <v>1066399.78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>68.9%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>167325.87</v>
+        <v>175994.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>796794.91</v>
+        <v>890404.91</v>
       </c>
       <c r="I4" t="n">
-        <v>800514</v>
+        <v>895804</v>
       </c>
       <c r="J4" t="n">
-        <v>-3720</v>
+        <v>-5400</v>
       </c>
       <c r="K4" t="n">
-        <v>607612</v>
+        <v>701222</v>
       </c>
     </row>
     <row r="5">
@@ -617,32 +617,32 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1536337.36</v>
+        <v>1558573.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>96.0%</t>
+          <t>97.4%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>359147.54</v>
+        <v>365747.54</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.5%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1177189.82</v>
+        <v>1192825.82</v>
       </c>
       <c r="I5" t="n">
-        <v>944366</v>
+        <v>960002</v>
       </c>
       <c r="J5" t="n">
         <v>232823</v>
       </c>
       <c r="K5" t="n">
-        <v>904543</v>
+        <v>899781</v>
       </c>
     </row>
     <row r="6">
@@ -703,15 +703,15 @@
         <v>2500000</v>
       </c>
       <c r="D7" t="n">
-        <v>1498813.799999999</v>
+        <v>1577089.09</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>63.1%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>65819</v>
+        <v>68819</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -719,16 +719,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1432994.799999999</v>
+        <v>1508270.09</v>
       </c>
       <c r="I7" t="n">
-        <v>583091</v>
+        <v>581489</v>
       </c>
       <c r="J7" t="n">
-        <v>849903</v>
+        <v>926781</v>
       </c>
       <c r="K7" t="n">
-        <v>1398804</v>
+        <v>1477080</v>
       </c>
     </row>
     <row r="8">
@@ -746,32 +746,32 @@
         <v>500000</v>
       </c>
       <c r="D8" t="n">
-        <v>186081.84</v>
+        <v>200698.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>37.2%</t>
+          <t>40.1%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>15876</v>
+        <v>16376</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.2%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>170205.84</v>
+        <v>184322.84</v>
       </c>
       <c r="I8" t="n">
-        <v>106014</v>
+        <v>105533</v>
       </c>
       <c r="J8" t="n">
-        <v>63791</v>
+        <v>78389</v>
       </c>
       <c r="K8" t="n">
-        <v>46253</v>
+        <v>45772</v>
       </c>
     </row>
     <row r="9">
@@ -789,11 +789,11 @@
         <v>600000</v>
       </c>
       <c r="D9" t="n">
-        <v>439884</v>
+        <v>449903</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>73.3%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -801,20 +801,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>428604</v>
+        <v>438623</v>
       </c>
       <c r="I9" t="n">
-        <v>25840</v>
+        <v>25859</v>
       </c>
       <c r="J9" t="n">
-        <v>402764</v>
+        <v>412764</v>
       </c>
       <c r="K9" t="n">
-        <v>106654</v>
+        <v>106673</v>
       </c>
     </row>
     <row r="10">
@@ -832,11 +832,11 @@
         <v>1000000</v>
       </c>
       <c r="D10" t="n">
-        <v>517343.33</v>
+        <v>590248.33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>51.7%</t>
+          <t>59.0%</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -844,20 +844,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>464024.33</v>
+        <v>536929.33</v>
       </c>
       <c r="I10" t="n">
-        <v>44501</v>
+        <v>44956</v>
       </c>
       <c r="J10" t="n">
-        <v>392334</v>
+        <v>464634</v>
       </c>
       <c r="K10" t="n">
-        <v>22882</v>
+        <v>68889</v>
       </c>
     </row>
     <row r="11">
@@ -875,32 +875,32 @@
         <v>1100000</v>
       </c>
       <c r="D11" t="n">
-        <v>759104.4700000001</v>
+        <v>766457.4700000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>69.0%</t>
+          <t>69.7%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>265839</v>
+        <v>265858</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>34.7%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>493265.4700000001</v>
+        <v>500599.4700000001</v>
       </c>
       <c r="I11" t="n">
-        <v>145720</v>
+        <v>132754</v>
       </c>
       <c r="J11" t="n">
-        <v>329670</v>
+        <v>349470</v>
       </c>
       <c r="K11" t="n">
-        <v>395909</v>
+        <v>403243</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>400000</v>
       </c>
       <c r="D12" t="n">
-        <v>125262.8</v>
+        <v>141376.8</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>31.3%</t>
+          <t>35.3%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>33.5%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>83312.47</v>
+        <v>99426.46999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>-4036</v>
+        <v>-3718</v>
       </c>
       <c r="J12" t="n">
-        <v>87348</v>
+        <v>103144</v>
       </c>
       <c r="K12" t="n">
-        <v>9025</v>
+        <v>9343</v>
       </c>
     </row>
     <row r="13">
@@ -961,11 +961,11 @@
         <v>500000</v>
       </c>
       <c r="D13" t="n">
-        <v>264787</v>
+        <v>274768</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>53.0%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -973,20 +973,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>219149</v>
+        <v>229130</v>
       </c>
       <c r="I13" t="n">
-        <v>57261</v>
+        <v>57242</v>
       </c>
       <c r="J13" t="n">
-        <v>161888</v>
+        <v>171888</v>
       </c>
       <c r="K13" t="n">
-        <v>61695</v>
+        <v>61676</v>
       </c>
     </row>
     <row r="14">
@@ -1004,32 +1004,32 @@
         <v>1900000</v>
       </c>
       <c r="D14" t="n">
-        <v>2080770.1</v>
+        <v>2122778.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>109.5%</t>
+          <t>111.7%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>314959</v>
+        <v>342899</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1765811.1</v>
+        <v>1779879.1</v>
       </c>
       <c r="I14" t="n">
-        <v>1361425</v>
+        <v>1347095</v>
       </c>
       <c r="J14" t="n">
-        <v>321417</v>
+        <v>349815</v>
       </c>
       <c r="K14" t="n">
-        <v>1489571</v>
+        <v>1465639</v>
       </c>
     </row>
     <row r="15">
@@ -1047,32 +1047,32 @@
         <v>1000000</v>
       </c>
       <c r="D15" t="n">
-        <v>1249760.04</v>
+        <v>1279877.04</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>125.0%</t>
+          <t>128.0%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>115766.59</v>
+        <v>116966.59</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1133993.45</v>
+        <v>1162910.45</v>
       </c>
       <c r="I15" t="n">
-        <v>214715</v>
+        <v>236434</v>
       </c>
       <c r="J15" t="n">
-        <v>897777</v>
+        <v>904975</v>
       </c>
       <c r="K15" t="n">
-        <v>485045</v>
+        <v>513962</v>
       </c>
     </row>
     <row r="16">
@@ -1090,32 +1090,32 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>614278.62</v>
+        <v>693127.48</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>68.3%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>66947</v>
+        <v>91447</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>547331.62</v>
+        <v>601680.48</v>
       </c>
       <c r="I16" t="n">
-        <v>124922</v>
+        <v>128031</v>
       </c>
       <c r="J16" t="n">
-        <v>369189</v>
+        <v>410089</v>
       </c>
       <c r="K16" t="n">
-        <v>63851</v>
+        <v>75900</v>
       </c>
     </row>
     <row r="17">
@@ -1133,11 +1133,11 @@
         <v>900000</v>
       </c>
       <c r="D17" t="n">
-        <v>306373</v>
+        <v>346889</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>38.5%</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1145,20 +1145,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>267523</v>
+        <v>308039</v>
       </c>
       <c r="I17" t="n">
-        <v>39153</v>
+        <v>69271</v>
       </c>
       <c r="J17" t="n">
-        <v>228370</v>
+        <v>238768</v>
       </c>
       <c r="K17" t="n">
-        <v>42323</v>
+        <v>62441</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
更新看板 10月27日 — KPI1383.5万(74.8%) 净流水1156.1万
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/导出_按分组.xlsx
+++ b/导出_按分组.xlsx
@@ -488,32 +488,32 @@
         <v>1450000</v>
       </c>
       <c r="D2" t="n">
-        <v>1017174.4</v>
+        <v>1151853.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>70.1%</t>
+          <t>79.4%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>166896.15</v>
+        <v>193989.15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>850278.2499999999</v>
+        <v>957864.2499999999</v>
       </c>
       <c r="I2" t="n">
-        <v>818005</v>
+        <v>942092</v>
       </c>
       <c r="J2" t="n">
-        <v>32272</v>
+        <v>15771</v>
       </c>
       <c r="K2" t="n">
-        <v>805426</v>
+        <v>903012</v>
       </c>
     </row>
     <row r="3">
@@ -531,32 +531,32 @@
         <v>1450000</v>
       </c>
       <c r="D3" t="n">
-        <v>442206.41</v>
+        <v>453012.4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30.5%</t>
+          <t>31.2%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>251409.07</v>
+        <v>275426.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>60.8%</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>190797.34</v>
+        <v>177586.33</v>
       </c>
       <c r="I3" t="n">
-        <v>151562</v>
+        <v>133371</v>
       </c>
       <c r="J3" t="n">
-        <v>39234</v>
+        <v>44214</v>
       </c>
       <c r="K3" t="n">
-        <v>203707</v>
+        <v>213996</v>
       </c>
     </row>
     <row r="4">
@@ -574,32 +574,32 @@
         <v>1400000</v>
       </c>
       <c r="D4" t="n">
-        <v>1066399.78</v>
+        <v>1125699.78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>76.2%</t>
+          <t>80.4%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>175994.87</v>
+        <v>176540.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>890404.91</v>
+        <v>949158.91</v>
       </c>
       <c r="I4" t="n">
-        <v>895804</v>
+        <v>954259</v>
       </c>
       <c r="J4" t="n">
-        <v>-5400</v>
+        <v>-5101</v>
       </c>
       <c r="K4" t="n">
-        <v>701222</v>
+        <v>759976</v>
       </c>
     </row>
     <row r="5">
@@ -617,11 +617,11 @@
         <v>1600000</v>
       </c>
       <c r="D5" t="n">
-        <v>1558573.36</v>
+        <v>1635045.36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>97.4%</t>
+          <t>102.2%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -629,20 +629,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1192825.82</v>
+        <v>1269297.82</v>
       </c>
       <c r="I5" t="n">
-        <v>960002</v>
+        <v>1016674</v>
       </c>
       <c r="J5" t="n">
-        <v>232823</v>
+        <v>252623</v>
       </c>
       <c r="K5" t="n">
-        <v>899781</v>
+        <v>927433</v>
       </c>
     </row>
     <row r="6">
@@ -660,32 +660,32 @@
         <v>1300000</v>
       </c>
       <c r="D6" t="n">
-        <v>549614</v>
+        <v>692174</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>42.3%</t>
+          <t>53.2%</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>44760</v>
+        <v>44940</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>504854</v>
+        <v>647234</v>
       </c>
       <c r="I6" t="n">
-        <v>503774</v>
+        <v>642194</v>
       </c>
       <c r="J6" t="n">
-        <v>1080</v>
+        <v>5040</v>
       </c>
       <c r="K6" t="n">
-        <v>445860</v>
+        <v>568440</v>
       </c>
     </row>
     <row r="7">
@@ -703,32 +703,32 @@
         <v>2500000</v>
       </c>
       <c r="D7" t="n">
-        <v>1577089.09</v>
+        <v>1590885.09</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>63.1%</t>
+          <t>63.6%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>68819</v>
+        <v>74819</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1508270.09</v>
+        <v>1516066.09</v>
       </c>
       <c r="I7" t="n">
-        <v>581489</v>
+        <v>591489</v>
       </c>
       <c r="J7" t="n">
-        <v>926781</v>
+        <v>924577</v>
       </c>
       <c r="K7" t="n">
-        <v>1477080</v>
+        <v>1490478</v>
       </c>
     </row>
     <row r="8">
@@ -746,11 +746,11 @@
         <v>500000</v>
       </c>
       <c r="D8" t="n">
-        <v>200698.84</v>
+        <v>211296.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>40.1%</t>
+          <t>42.3%</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -758,17 +758,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>184322.84</v>
+        <v>194920.84</v>
       </c>
       <c r="I8" t="n">
         <v>105533</v>
       </c>
       <c r="J8" t="n">
-        <v>78389</v>
+        <v>88987</v>
       </c>
       <c r="K8" t="n">
         <v>45772</v>
@@ -789,32 +789,32 @@
         <v>600000</v>
       </c>
       <c r="D9" t="n">
-        <v>449903</v>
+        <v>516522</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>86.1%</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11280</v>
+        <v>20280</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.5%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>438623</v>
+        <v>496242</v>
       </c>
       <c r="I9" t="n">
-        <v>25859</v>
+        <v>45678</v>
       </c>
       <c r="J9" t="n">
-        <v>412764</v>
+        <v>450564</v>
       </c>
       <c r="K9" t="n">
-        <v>106673</v>
+        <v>163292</v>
       </c>
     </row>
     <row r="10">
@@ -832,32 +832,32 @@
         <v>1000000</v>
       </c>
       <c r="D10" t="n">
-        <v>590248.33</v>
+        <v>668540.33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>66.9%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>53319</v>
+        <v>61319</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>9.2%</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>536929.33</v>
+        <v>607221.33</v>
       </c>
       <c r="I10" t="n">
-        <v>44956</v>
+        <v>59956</v>
       </c>
       <c r="J10" t="n">
-        <v>464634</v>
+        <v>519926</v>
       </c>
       <c r="K10" t="n">
-        <v>68889</v>
+        <v>68983</v>
       </c>
     </row>
     <row r="11">
@@ -875,7 +875,7 @@
         <v>1100000</v>
       </c>
       <c r="D11" t="n">
-        <v>766457.4700000001</v>
+        <v>767192.6200000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -883,24 +883,24 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>265858</v>
+        <v>267838</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>34.7%</t>
+          <t>34.9%</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>500599.4700000001</v>
+        <v>499354.6200000001</v>
       </c>
       <c r="I11" t="n">
-        <v>132754</v>
+        <v>131429</v>
       </c>
       <c r="J11" t="n">
         <v>349470</v>
       </c>
       <c r="K11" t="n">
-        <v>403243</v>
+        <v>401400</v>
       </c>
     </row>
     <row r="12">
@@ -918,11 +918,11 @@
         <v>400000</v>
       </c>
       <c r="D12" t="n">
-        <v>141376.8</v>
+        <v>149089.8</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>37.3%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -930,20 +930,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>29.7%</t>
+          <t>28.1%</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>99426.46999999999</v>
+        <v>107139.47</v>
       </c>
       <c r="I12" t="n">
-        <v>-3718</v>
+        <v>-2801</v>
       </c>
       <c r="J12" t="n">
-        <v>103144</v>
+        <v>109940</v>
       </c>
       <c r="K12" t="n">
-        <v>9343</v>
+        <v>9862</v>
       </c>
     </row>
     <row r="13">
@@ -961,32 +961,32 @@
         <v>500000</v>
       </c>
       <c r="D13" t="n">
-        <v>274768</v>
+        <v>294568</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>58.9%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45638</v>
+        <v>49238</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>229130</v>
+        <v>245330</v>
       </c>
       <c r="I13" t="n">
-        <v>57242</v>
+        <v>77042</v>
       </c>
       <c r="J13" t="n">
-        <v>171888</v>
+        <v>168288</v>
       </c>
       <c r="K13" t="n">
-        <v>61676</v>
+        <v>81476</v>
       </c>
     </row>
     <row r="14">
@@ -1004,32 +1004,32 @@
         <v>1900000</v>
       </c>
       <c r="D14" t="n">
-        <v>2122778.1</v>
+        <v>2142791.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>111.7%</t>
+          <t>112.8%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>342899</v>
+        <v>359718</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1779879.1</v>
+        <v>1783073.1</v>
       </c>
       <c r="I14" t="n">
-        <v>1347095</v>
+        <v>1334293</v>
       </c>
       <c r="J14" t="n">
-        <v>349815</v>
+        <v>365811</v>
       </c>
       <c r="K14" t="n">
-        <v>1465639</v>
+        <v>1452837</v>
       </c>
     </row>
     <row r="15">
@@ -1047,32 +1047,32 @@
         <v>1000000</v>
       </c>
       <c r="D15" t="n">
-        <v>1279877.04</v>
+        <v>1312030.18</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>128.0%</t>
+          <t>131.2%</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>116966.59</v>
+        <v>168085.59</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1162910.45</v>
+        <v>1143944.59</v>
       </c>
       <c r="I15" t="n">
-        <v>236434</v>
+        <v>209412</v>
       </c>
       <c r="J15" t="n">
-        <v>904975</v>
+        <v>913031</v>
       </c>
       <c r="K15" t="n">
-        <v>513962</v>
+        <v>489700</v>
       </c>
     </row>
     <row r="16">
@@ -1090,11 +1090,11 @@
         <v>900000</v>
       </c>
       <c r="D16" t="n">
-        <v>693127.48</v>
+        <v>733442.48</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>77.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1102,20 +1102,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>601680.48</v>
+        <v>641995.48</v>
       </c>
       <c r="I16" t="n">
-        <v>128031</v>
+        <v>134846</v>
       </c>
       <c r="J16" t="n">
-        <v>410089</v>
+        <v>443589</v>
       </c>
       <c r="K16" t="n">
-        <v>75900</v>
+        <v>75919</v>
       </c>
     </row>
     <row r="17">
@@ -1133,32 +1133,32 @@
         <v>900000</v>
       </c>
       <c r="D17" t="n">
-        <v>346889</v>
+        <v>358083</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>39.8%</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>38850</v>
+        <v>53269</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>308039</v>
+        <v>304814</v>
       </c>
       <c r="I17" t="n">
-        <v>69271</v>
+        <v>69650</v>
       </c>
       <c r="J17" t="n">
-        <v>238768</v>
+        <v>235164</v>
       </c>
       <c r="K17" t="n">
-        <v>62441</v>
+        <v>62422</v>
       </c>
     </row>
     <row r="18">

</xml_diff>